<commit_message>
Mise à jour des ressources FSH 0679381b966dd91070216c1828d6cfa13481f39f
</commit_message>
<xml_diff>
--- a/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
+++ b/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-01-02T14:56:23+00:00</t>
+    <t>2025-01-06T16:20:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -436,7 +436,7 @@
 </t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J01-XdsAuthorSpecialty-CISIS/FHIR/JDV-J01-XdsAuthorSpecialty-CISIS/</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J01-XdsAuthorSpecialty-CISIS/FHIR/JDV-J01-XdsAuthorSpecialty-CISIS</t>
   </si>
   <si>
     <t>AssignedAuthor.addr</t>
@@ -456,21 +456,21 @@
     <t>AssignedAuthor.assignedPerson</t>
   </si>
   <si>
-    <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/Person
+    <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/Person {https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-core-person}
 </t>
   </si>
   <si>
     <t>AssignedAuthor.assignedAuthoringDevice</t>
   </si>
   <si>
-    <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/AuthoringDevice
+    <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/AuthoringDevice {https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-core-authoring-device}
 </t>
   </si>
   <si>
     <t>AssignedAuthor.representedOrganization</t>
   </si>
   <si>
-    <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/Organization
+    <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/Organization {https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-core-represented-organization}
 </t>
   </si>
 </sst>
@@ -801,7 +801,7 @@
     <col min="23" max="23" width="19.03515625" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="18.859375" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="21.57421875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="98.36328125" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="97.74609375" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="6.34765625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="22.71875" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="20.59375" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
Correction suite au review du Nidal sur la partie CDA 5af7517b66330f13995287792f071b14958c1eb0
</commit_message>
<xml_diff>
--- a/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
+++ b/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="816" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="151">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-01-15T14:08:36+00:00</t>
+    <t>2025-01-17T15:05:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -317,6 +317,10 @@
     <t>InfrastructureRoot.typeId</t>
   </si>
   <si>
+    <t xml:space="preserve">II-1:An II instance must have either a root or an nullFlavor. {root.exists() or nullFlavor.exists()}
+</t>
+  </si>
+  <si>
     <t>AssignedAuthor.typeId.nullFlavor</t>
   </si>
   <si>
@@ -416,10 +420,20 @@
     <t>AssignedAuthor.id.root</t>
   </si>
   <si>
+    <t>- Pour un professionnel : '1.2.250.1.71.4.2.1'
+- Pour le patient/usager : OID de l'autorité d'affectation de l'INS
+- Pour un système de structure : '1.2.250.1.71.4.2.1' 
+- Pour un SNR : OID de l'éditeur 
+- Pour le DP : '1.2.250.1.71.4.2.1'</t>
+  </si>
+  <si>
     <t>A unique identifier that guarantees the global uniqueness of the instance identifier. The root alone may be the entire instance identifier.</t>
   </si>
   <si>
     <t>AssignedAuthor.id.extension</t>
+  </si>
+  <si>
+    <t>Valeur de l’identifiant</t>
   </si>
   <si>
     <t>AssignedAuthor.sdtcIdentifiedBy</t>
@@ -1327,7 +1341,7 @@
         <v>74</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>74</v>
+        <v>99</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>74</v>
@@ -1335,10 +1349,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1436,17 +1450,17 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E7" t="s" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F7" t="s" s="2">
         <v>80</v>
@@ -1464,11 +1478,11 @@
         <v>74</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L7" s="2"/>
       <c r="M7" t="s" s="2">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1519,7 +1533,7 @@
         <v>74</v>
       </c>
       <c r="AF7" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>80</v>
@@ -1539,17 +1553,17 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E8" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F8" t="s" s="2">
         <v>80</v>
@@ -1567,11 +1581,11 @@
         <v>74</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L8" s="2"/>
       <c r="M8" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -1622,7 +1636,7 @@
         <v>74</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>80</v>
@@ -1642,17 +1656,17 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E9" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F9" t="s" s="2">
         <v>75</v>
@@ -1670,11 +1684,11 @@
         <v>74</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="L9" s="2"/>
       <c r="M9" t="s" s="2">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1683,7 +1697,7 @@
       </c>
       <c r="Q9" s="2"/>
       <c r="R9" t="s" s="2">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="S9" t="s" s="2">
         <v>74</v>
@@ -1725,7 +1739,7 @@
         <v>74</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>80</v>
@@ -1745,17 +1759,17 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B10" t="s" s="2">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E10" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F10" t="s" s="2">
         <v>75</v>
@@ -1773,11 +1787,11 @@
         <v>74</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L10" s="2"/>
       <c r="M10" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1828,7 +1842,7 @@
         <v>74</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>80</v>
@@ -1848,10 +1862,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -1878,7 +1892,7 @@
       </c>
       <c r="L11" s="2"/>
       <c r="M11" t="s" s="2">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -1929,7 +1943,7 @@
         <v>74</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>80</v>
@@ -1949,10 +1963,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -1986,7 +2000,7 @@
       </c>
       <c r="Q12" s="2"/>
       <c r="R12" t="s" s="2">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="S12" t="s" s="2">
         <v>74</v>
@@ -2008,7 +2022,7 @@
       </c>
       <c r="Y12" s="2"/>
       <c r="Z12" t="s" s="2">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="AA12" t="s" s="2">
         <v>74</v>
@@ -2026,7 +2040,7 @@
         <v>74</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>80</v>
@@ -2046,10 +2060,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2125,7 +2139,7 @@
         <v>74</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>75</v>
@@ -2145,10 +2159,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2246,23 +2260,23 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E15" t="s" s="2">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="F15" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>74</v>
@@ -2274,11 +2288,11 @@
         <v>74</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="L15" s="2"/>
       <c r="M15" t="s" s="2">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2329,7 +2343,7 @@
         <v>74</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>80</v>
@@ -2349,23 +2363,23 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E16" t="s" s="2">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F16" t="s" s="2">
         <v>80</v>
       </c>
       <c r="G16" t="s" s="2">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H16" t="s" s="2">
         <v>74</v>
@@ -2377,11 +2391,11 @@
         <v>74</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="L16" s="2"/>
       <c r="M16" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -2432,7 +2446,7 @@
         <v>74</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>80</v>
@@ -2452,20 +2466,20 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E17" t="s" s="2">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F17" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G17" t="s" s="2">
         <v>75</v>
@@ -2480,11 +2494,13 @@
         <v>74</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>112</v>
-      </c>
-      <c r="L17" s="2"/>
+        <v>113</v>
+      </c>
+      <c r="L17" t="s" s="2">
+        <v>132</v>
+      </c>
       <c r="M17" t="s" s="2">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2535,7 +2551,7 @@
         <v>74</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>80</v>
@@ -2555,20 +2571,20 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
         <v>74</v>
       </c>
       <c r="E18" t="s" s="2">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F18" t="s" s="2">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="G18" t="s" s="2">
         <v>75</v>
@@ -2583,11 +2599,13 @@
         <v>74</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>102</v>
-      </c>
-      <c r="L18" s="2"/>
+        <v>103</v>
+      </c>
+      <c r="L18" t="s" s="2">
+        <v>135</v>
+      </c>
       <c r="M18" t="s" s="2">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="N18" s="2"/>
       <c r="O18" s="2"/>
@@ -2638,7 +2656,7 @@
         <v>74</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>80</v>
@@ -2658,10 +2676,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2684,7 +2702,7 @@
         <v>74</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
@@ -2737,7 +2755,7 @@
         <v>74</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>80</v>
@@ -2757,10 +2775,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2783,7 +2801,7 @@
         <v>74</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="L20" s="2"/>
       <c r="M20" s="2"/>
@@ -2816,7 +2834,7 @@
       </c>
       <c r="Y20" s="2"/>
       <c r="Z20" t="s" s="2">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>74</v>
@@ -2834,7 +2852,7 @@
         <v>74</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>80</v>
@@ -2854,10 +2872,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2880,7 +2898,7 @@
         <v>74</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="L21" s="2"/>
       <c r="M21" s="2"/>
@@ -2933,7 +2951,7 @@
         <v>74</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>80</v>
@@ -2953,10 +2971,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -2979,7 +2997,7 @@
         <v>74</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="L22" s="2"/>
       <c r="M22" s="2"/>
@@ -3032,7 +3050,7 @@
         <v>74</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>80</v>
@@ -3052,10 +3070,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3078,7 +3096,7 @@
         <v>74</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
@@ -3131,7 +3149,7 @@
         <v>74</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>80</v>
@@ -3151,10 +3169,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3177,7 +3195,7 @@
         <v>74</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
@@ -3230,7 +3248,7 @@
         <v>74</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -3250,10 +3268,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3276,7 +3294,7 @@
         <v>74</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -3329,7 +3347,7 @@
         <v>74</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
Ajout des descriptions manquantes dans les ressourcesCDA+Corrections suite à la revue b45ce25d09bbd54f796cdfabf02779e21d8bbcf1
</commit_message>
<xml_diff>
--- a/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
+++ b/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="818" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="825" uniqueCount="158">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-03T10:34:19+00:00</t>
+    <t>2025-02-05T14:18:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -406,6 +406,14 @@
   </si>
   <si>
     <t>AssignedAuthor.id</t>
+  </si>
+  <si>
+    <t>Identifiant de l’auteur : 
+- Obligatoire pour un professionnel 
+- Obligatoire pour le patient/usager 
+- Obligatoire pour un système de structure 
+- Obligatoire pour un SNR 
+- Obligatoire pour le DP</t>
   </si>
   <si>
     <t>AssignedAuthor.id.nullFlavor</t>
@@ -450,6 +458,14 @@
 </t>
   </si>
   <si>
+    <t>Profession / savoir-faire ou rôle : 
+- Obligatoire pour un professionnel 
+- Ne pas utiliser pour le patient/usager 
+- Obligatoire pour un système de structure 
+- Obligatoire pour un SNR 
+- Obligatoire pour le DP</t>
+  </si>
+  <si>
     <t>https://mos.esante.gouv.fr/NOS/JDV_J01-XdsAuthorSpecialty-CISIS/FHIR/JDV-J01-XdsAuthorSpecialty-CISIS</t>
   </si>
   <si>
@@ -460,6 +476,9 @@
 </t>
   </si>
   <si>
+    <t>Adresse géopostale de l’auteur</t>
+  </si>
+  <si>
     <t>AssignedAuthor.telecom</t>
   </si>
   <si>
@@ -467,6 +486,9 @@
 </t>
   </si>
   <si>
+    <t>Coordonnées télécom de l’auteur</t>
+  </si>
+  <si>
     <t>AssignedAuthor.assignedPerson</t>
   </si>
   <si>
@@ -474,6 +496,14 @@
 </t>
   </si>
   <si>
+    <t>Identité de l’auteur :  
+- Obligatoire pour un professionnel 
+- Obligatoire pour le patient/usager 
+- Ne pas utiliser pour un système de structure 
+- Ne pas utiliser pour un SNR 
+- Ne pas utiliser pour le DP</t>
+  </si>
+  <si>
     <t>AssignedAuthor.assignedAuthoringDevice</t>
   </si>
   <si>
@@ -481,11 +511,28 @@
 </t>
   </si>
   <si>
+    <t>Informations complémentaires si l’auteur est 
+un système :
+- Ne pas utiliser pour un professionnel 
+- Ne pas utiliser pour le patient/usager 
+- Obligatoire pour un système de structure 
+- Obligatoire pour un SNR 
+- Obligatoire pour le DP</t>
+  </si>
+  <si>
     <t>AssignedAuthor.representedOrganization</t>
   </si>
   <si>
     <t xml:space="preserve">http://hl7.org/cda/stds/core/StructureDefinition/Organization {https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-core-represented-organization}
 </t>
+  </si>
+  <si>
+    <t>Structure correspondante : 
+- Obligatoire pour un professionnel 
+- Ne pas utiliser pour le patient/usager 
+- Obligatoire pour un système de structure 
+- Obligatoire pour un SNR 
+- Obligatoire pour le DP</t>
   </si>
 </sst>
 </file>
@@ -2088,7 +2135,9 @@
       <c r="K13" t="s" s="2">
         <v>96</v>
       </c>
-      <c r="L13" s="2"/>
+      <c r="L13" t="s" s="2">
+        <v>128</v>
+      </c>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2159,10 +2208,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2260,10 +2309,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -2363,10 +2412,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2466,10 +2515,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2497,10 +2546,10 @@
         <v>113</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2571,10 +2620,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2602,7 +2651,7 @@
         <v>103</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M18" t="s" s="2">
         <v>119</v>
@@ -2676,10 +2725,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2702,7 +2751,7 @@
         <v>74</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
@@ -2755,7 +2804,7 @@
         <v>74</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>80</v>
@@ -2775,10 +2824,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -2801,9 +2850,11 @@
         <v>74</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>139</v>
-      </c>
-      <c r="L20" s="2"/>
+        <v>140</v>
+      </c>
+      <c r="L20" t="s" s="2">
+        <v>141</v>
+      </c>
       <c r="M20" s="2"/>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2834,7 +2885,7 @@
       </c>
       <c r="Y20" s="2"/>
       <c r="Z20" t="s" s="2">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>74</v>
@@ -2852,7 +2903,7 @@
         <v>74</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>80</v>
@@ -2872,10 +2923,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2898,9 +2949,11 @@
         <v>74</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>142</v>
-      </c>
-      <c r="L21" s="2"/>
+        <v>144</v>
+      </c>
+      <c r="L21" t="s" s="2">
+        <v>145</v>
+      </c>
       <c r="M21" s="2"/>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -2951,7 +3004,7 @@
         <v>74</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>80</v>
@@ -2971,10 +3024,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -2997,9 +3050,11 @@
         <v>74</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="L22" s="2"/>
+        <v>147</v>
+      </c>
+      <c r="L22" t="s" s="2">
+        <v>148</v>
+      </c>
       <c r="M22" s="2"/>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3050,7 +3105,7 @@
         <v>74</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>80</v>
@@ -3070,10 +3125,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3096,9 +3151,11 @@
         <v>74</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>146</v>
-      </c>
-      <c r="L23" s="2"/>
+        <v>150</v>
+      </c>
+      <c r="L23" t="s" s="2">
+        <v>151</v>
+      </c>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3149,7 +3206,7 @@
         <v>74</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>80</v>
@@ -3169,10 +3226,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3195,9 +3252,11 @@
         <v>74</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="L24" s="2"/>
+        <v>153</v>
+      </c>
+      <c r="L24" t="s" s="2">
+        <v>154</v>
+      </c>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3248,7 +3307,7 @@
         <v>74</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>80</v>
@@ -3268,10 +3327,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -3294,9 +3353,11 @@
         <v>74</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>150</v>
-      </c>
-      <c r="L25" s="2"/>
+        <v>156</v>
+      </c>
+      <c r="L25" t="s" s="2">
+        <v>157</v>
+      </c>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3347,7 +3408,7 @@
         <v>74</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>80</v>

</xml_diff>

<commit_message>
Corrections suite à la revue 7c42c3f0bc2805c35b1bff13a8a7fc83a375ef8b
</commit_message>
<xml_diff>
--- a/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
+++ b/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-05T14:18:33+00:00</t>
+    <t>2025-02-05T15:17:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -511,8 +511,7 @@
 </t>
   </si>
   <si>
-    <t>Informations complémentaires si l’auteur est 
-un système :
+    <t>Informations complémentaires si l’auteur est un système :
 - Ne pas utiliser pour un professionnel 
 - Ne pas utiliser pour le patient/usager 
 - Obligatoire pour un système de structure 

</xml_diff>

<commit_message>
Suppression des pages inutilisées et MAJ des descriptions de l'ensemble des éléments 0c1aeb37043c78d70f95d48ea9d328366548218a
</commit_message>
<xml_diff>
--- a/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
+++ b/SBM-initDocIG/ig/StructureDefinition-fr-core-assigned-author.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-05T15:35:39+00:00</t>
+    <t>2025-02-06T13:21:10+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -81,7 +81,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>assignedAuthor contient les éléments permettant de décrire l’auteur.</t>
+    <t>L'élément de l'en-tête du CDA assignedAuthor contient les éléments permettant de décrire l’auteur.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>